<commit_message>
Add meeting notes document for project tracking
</commit_message>
<xml_diff>
--- a/tableau arbitrage.xlsx
+++ b/tableau arbitrage.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="arbitrages" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="76">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -178,69 +178,166 @@
     <t xml:space="preserve">Acteurs présents</t>
   </si>
   <si>
+    <t xml:space="preserve">Durée (h)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Points clés abordés</t>
   </si>
   <si>
+    <t xml:space="preserve">Point initial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Marjolaine Fabien</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lancement du projet rôle AMOA historique PPE premières réflexions techniques modèle de données architecture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avancement projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préparation réunion de lancement cadrage du projet organisation des rôles gouvernance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Marjolaine Emma Stéphane salomé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Présentation Hydroscope objectifs gouvernance enjeux ressource en eau définition des phases du projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Débrief projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Marjolaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suivi de l’avancement gestion du temps organisation des tâches outils de pilotage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pré-COPRO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Préparation du COPRO cadrage stratégique organisation des ateliers identification des partenaires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Marjolaine Stéphane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gouvernance du projet validation du cadrage fonctionnel rôle des interfaces analyse multicritère organisation des ateliers métiers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clarification des interfaces expert vs partenaire accès aux données importance de l’analyse multicritère gestion des droits utilisateurs</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cadrage fonctionnel</t>
   </si>
   <si>
-    <t xml:space="preserve">Hugo; Marjolaine; Stéphane</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Structuration des indicateurs; définition des familles (enjeux, pressions, vulnérabilité); clarification des livrables; analyse multicritère; organisation des données</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avancement projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hugo; Marjolaine ; Fabien</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clarification des interfaces (expert vs partenaire); accès aux données; importance de l’analyse multicritère; gestion des droits utilisateurs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gouvernance du projet; validation du cadrage fonctionnel; rôle des interfaces; analyse multicritère; organisation des ateliers métiers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pré-COPRO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préparation du COPRO; cadrage stratégique; organisation des ateliers; identification des partenaires</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Débrief projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hugo; Marjolaine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suivi de l’avancement; gestion du temps; organisation des tâches; outils de pilotage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hugo; Marjolaine; Emma; Stéphane; autres</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Présentation Hydroscope; objectifs; gouvernance; enjeux ressource en eau; définition des phases du projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Préparation réunion de lancement; cadrage du projet; organisation des rôles; gouvernance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Point initial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lancement du projet; rôle AMOA; historique PPE; premières réflexions techniques (modèle de données; architecture)</t>
+    <t xml:space="preserve">Structuration des indicateurs définition des familles enjeux pressions vulnérabilité clarification des livrables organisation des données</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilatérale DAVAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Échange sur les attentes DAVAR validation des orientations indicateurs organisation des données et du cadrage fonctionnel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atelier métiers partenaires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Marjolaine partenaires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recueil des besoins métiers retours des acteurs identification des usages et des attentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point gestion de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suivi de l’avancement coordination des travaux organisation des prochaines étapes du projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilatérales DIMENC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Marjolaine DIMENC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Échanges sur les données disponibles identification des besoins acteurs cadrage des usages potentiels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point sur l’avancement préparation des bilatérales suivi des échanges partenaires annulation DASS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réunion présentation Hydroscope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Marjolaine Stéphane Province Sud Mairie Thio autres partenaires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Présentation du projet aux partenaires recueil des premiers retours organisation des bilatérales clarification des attentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilatérale Province Sud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Marjolaine Province Sud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discussion sur les indicateurs et la méthode analyse multicritère besoins spécifiques Province Sud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilatérale SIVOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Marjolaine SIVOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Échange sur les besoins terrain données disponibles contraintes opérationnelles usages attendus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilatérale EAUNC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Marjolaine EAUNC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Échange sur les données techniques modalités d’intégration contraintes liées aux données et aux usages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COPRO point indicateur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avancement des fiches indicateurs validation des orientations préparation des livrables indicateurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilatérale CDE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Marjolaine CDE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discussion sur les besoins en données contraintes métiers attentes vis-à-vis de l’outil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Point d’avancement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suivi global du projet ajustement des priorités organisation de la suite des travaux</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
-    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="167" formatCode="0.00"/>
+    <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -320,7 +417,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -341,7 +438,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -365,37 +470,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -475,9 +580,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="45.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="24.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="24.06"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -621,166 +726,431 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="49.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="42.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="5" width="26.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="5" t="s">
         <v>26</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>46076</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>46091</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>46094</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>46098</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>46115</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>46121</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>46126</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>46136</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="0" t="s">
+      <c r="C9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>46136</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>46163</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>46170</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>46175</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>46181</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>46197</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>46205</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>46126</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="B4" s="5" t="n">
-        <v>46121</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" s="0" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>46115</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="0" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>46098</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="E21" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>46094</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="E7" s="0" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>46091</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" s="0" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>46076</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="0" t="s">
-        <v>43</v>
+      <c r="F21" s="1" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>